<commit_message>
test: keep the prescription edit inside the visit test
</commit_message>
<xml_diff>
--- a/smart-healthcare-frontend/test-cases/test-cases.xlsx
+++ b/smart-healthcare-frontend/test-cases/test-cases.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2836,108 +2836,61 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Verify that the doctor can change a prescription he already wrote</t>
+          <t>Verify that Cancel in the ConfirmDialog keeps the prescription</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>The doctor dr_smith is logged in from the before step. The prescription with the diagnosis Seasonal flu is already there.</t>
+          <t>The doctor dr_smith is logged in from the before step. The doctor already wrote prescriptions.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Prescriptions page
-2. Edit the prescription
-3. Change the diagnosis
-4. Change it back</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>Diagnosis Seasonal flu, then a diagnosis with a unique number</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>A toast reads "Prescription saved.", the row shows the new diagnosis, and after the change back the old diagnosis is there again.</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="62" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>TC-052</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Doctor</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Verify Doctor Prescriptions</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Verify that Cancel in the ConfirmDialog keeps the prescription</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>The doctor dr_smith is logged in from the before step. The doctor already wrote prescriptions.</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1. Open the Prescriptions page
 2. Click Delete prescription on the first row
 3. Click Cancel</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>No data</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>The dialog closes and the table still has the same number of rows.</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54" ht="62" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>TC-053</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="62" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TC-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Doctor</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Verify Doctor Profile</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Verify that the doctor can change his own specialty</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>The doctor dr_smith is logged in from the before step.</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1. Open the Profile page
 2. Click Edit Profile
@@ -2945,14 +2898,58 @@
 4. Change it back to Cardiology</t>
         </is>
       </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>A specialty with a unique number, then Cardiology</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>A toast reads "Profile saved." and the new specialty is shown, then Cardiology is shown again.</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="62" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>TC-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Verify Patient Access</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Verify that a patient can not open an admin page</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>The patient john_doe is logged in from the before step.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Doctors adress directly</t>
+        </is>
+      </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>A specialty with a unique number, then Cardiology</t>
+          <t>/dashboard/doctors</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>A toast reads "Profile saved." and the new specialty is shown, then Cardiology is shown again.</t>
+          <t>The app sends the patient back to his own dashboard.</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -2976,7 +2973,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Verify that a patient can not open an admin page</t>
+          <t>Verify that a patient can not open a doctor page</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -2986,12 +2983,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>1. Open the Doctors adress directly</t>
+          <t>1. Open the doctor work hours adress directly</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>/dashboard/doctors</t>
+          <t>/dashboard/availability</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3015,64 +3012,20 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Verify Patient Access</t>
+          <t>Verify Patient Appointments</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Verify that a patient can not open a doctor page</t>
+          <t>Verify that the patient can book an appointment, cancel it and delete it</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>The patient john_doe is logged in from the before step.</t>
+          <t>The patient john_doe is logged in from the before step. The appointment the test needs is booked in the before step.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the doctor work hours adress directly</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>/dashboard/availability</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>The app sends the patient back to his own dashboard.</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="62" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>TC-056</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Verify Patient Appointments</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Verify that the patient can book an appointment, cancel it and delete it</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>The patient john_doe is logged in from the before step. The appointment the test needs is booked in the before step.</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Book an appointment
@@ -3080,92 +3033,92 @@
 4. Delete it</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Dr. Sarah Smith, a Monday four weeks ahead, the first free time, a reason with a unique number</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>A toast reads "Appointment booked." and the row is Scheduled, then "Appointment cancelled." and the row is Cancelled, then "Appointment deleted." and the row is gone.</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58" ht="62" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>TC-057</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="62" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>TC-056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Verify that the booking form does not book before a doctor and a date are picked</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Click Book Appointment
 3. Look at the Book Appointment button</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>No doctor and no date picked</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>The Book Appointment button is disabled and Cancel closes the drawer.</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59" ht="62" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>TC-058</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58" ht="62" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TC-057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Verify that a day the doctor does not work offers no times</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step. The doctor does not work on Sunday.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Click Book Appointment
@@ -3173,46 +3126,46 @@
 4. Pick a Sunday</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>Dr. Sarah Smith, a Sunday four weeks ahead</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>The Time field reads "Doctor not available on SUNDAY" and the Book Appointment button stays disabled.</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60" ht="62" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>TC-059</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="62" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>TC-058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Verify that Cancel throws away what was typed in the booking form</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Click Book Appointment
@@ -3221,46 +3174,46 @@
 5. Open the form again</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>A reason with a unique number</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>The drawer closes, and when it is opened again the reason is empty.</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61" ht="62" customHeight="1">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>TC-060</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60" ht="62" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>TC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Verify that Keep it in the ConfirmDialog keeps the appointment</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step. The appointment is booked in the before step.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Book an appointment
@@ -3269,46 +3222,46 @@
 5. Remove the appointment</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>Dr. Sarah Smith, a Monday five weeks ahead</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>The dialog names the doctor, the date and the time, and after Keep it the row is still Scheduled.</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62" ht="62" customHeight="1">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>TC-061</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="62" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>TC-060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Verify that a time that is already booked is not offered again</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step. The appointment is booked in the before step.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Book the first free time
@@ -3316,14 +3269,59 @@
 4. Remove the appointment</t>
         </is>
       </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Sarah Smith, a Monday seven weeks ahead</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>The first free time is not the one that was just booked.</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62" ht="62" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>TC-061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Verify Patient Appointments</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Verify that the appointments calendar shows a column for every day of the week</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>The patient john_doe is logged in from the before step.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Appointments page
+2. Switch to the calendar view</t>
+        </is>
+      </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Dr. Sarah Smith, a Monday seven weeks ahead</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>The first free time is not the one that was just booked.</t>
+          <t>The calendar shows the seven days of the week and the week label.</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3347,7 +3345,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Verify that the appointments calendar shows a column for every day of the week</t>
+          <t>Verify that the patient can walk to the next week and come back</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3356,51 +3354,6 @@
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Appointments page
-2. Switch to the calendar view</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>No data</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>The calendar shows the seven days of the week and the week label.</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64" ht="62" customHeight="1">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>TC-063</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Verify Patient Appointments</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>Verify that the patient can walk to the next week and come back</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>The patient john_doe is logged in from the before step.</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Switch to the calendar view
@@ -3408,46 +3361,46 @@
 4. Click This week</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>No data</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>The week label changes when the week is changed and comes back to the same week after This week.</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65" ht="62" customHeight="1">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>TC-064</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64" ht="62" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>TC-063</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Verify that the patient can open the details of an appointment</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step. The appointment is booked in the before step.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Book an appointment
@@ -3456,52 +3409,96 @@
 5. Remove the appointment</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>Dr. Sarah Smith, a Monday six weeks ahead</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>The drawer shows Appointment Details with the doctor and the reason that were booked.</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66" ht="62" customHeight="1">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>TC-065</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65" ht="62" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>TC-064</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Appointments</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Verify that the view the patient picked is still there after a reload</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step.</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. Open the Appointments page
 2. Switch to the list view
 3. Reload the page</t>
         </is>
       </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>The list view is still the one that is shown after the reload.</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66" ht="62" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>TC-065</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Verify Patient Prescriptions</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Verify that the patient can see the prescriptions written for him</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>The patient john_doe is logged in from the before step. The patient already has prescriptions.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Prescriptions page</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
           <t>No data</t>
@@ -3509,7 +3506,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>The list view is still the one that is shown after the reload.</t>
+          <t>The heading reads My Prescriptions and the table has rows.</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -3533,7 +3530,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Verify that the patient can see the prescriptions written for him</t>
+          <t>Verify that the patient can open the details of a prescription</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -3542,56 +3539,56 @@
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Prescriptions page</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>No data</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>The heading reads My Prescriptions and the table has rows.</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68" ht="62" customHeight="1">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>TC-067</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Verify Patient Prescriptions</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Verify that the patient can open the details of a prescription</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>The patient john_doe is logged in from the before step. The patient already has prescriptions.</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. Open the Prescriptions page
 2. Click View details on the first row
 3. Close the drawer</t>
         </is>
       </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>The drawer opens with the title Prescription Details and closes again.</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68" ht="62" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>TC-067</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Verify Patient Medical Record</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Verify that the patient can see his own medical record</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>The patient john_doe is logged in from the before step. The patient already has visits and prescriptions.</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Medical Record page</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
           <t>No data</t>
@@ -3599,7 +3596,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>The drawer opens with the title Prescription Details and closes again.</t>
+          <t>The heading reads My Medical Record, the patient name is shown and the timeline has items.</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
@@ -3623,7 +3620,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Verify that the patient can see his own medical record</t>
+          <t>Verify that the record can be filtered down to one kind of item</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3632,96 +3629,52 @@
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Medical Record page</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>No data</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>The heading reads My Medical Record, the patient name is shown and the timeline has items.</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70" ht="62" customHeight="1">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>TC-069</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Verify Patient Medical Record</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Verify that the record can be filtered down to one kind of item</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>The patient john_doe is logged in from the before step. The patient already has visits and prescriptions.</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. Open the Medical Record page
 2. Click the Visits filter
 3. Click the Prescriptions filter</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>No data</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>The Visits filter leaves only the visits and the Prescriptions filter leaves only the prescriptions.</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71" ht="62" customHeight="1">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>TC-070</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70" ht="62" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>TC-069</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Medical Record</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Verify that the patient can open a visit from his record</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step. The patient already has visits.</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. Open the Medical Record page
 2. Click the Visits filter
@@ -3729,46 +3682,46 @@
 4. Close the drawer</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>No data</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>The drawer opens with the title Appointment Details and closes again.</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72" ht="62" customHeight="1">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>TC-071</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71" ht="62" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TC-070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Verify Patient Profile</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>Verify that the patient can change his phone and address</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe is logged in from the before step.</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>1. Open the Profile page
 2. Click Edit Profile
@@ -3776,14 +3729,58 @@
 4. Change them back</t>
         </is>
       </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>0799999999 and Irbid, Jordan, then 0791234567 and Amman, Jordan</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>A toast reads "Profile saved." and the new phone and adress are shown, then the old ones are shown again.</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72" ht="62" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>TC-071</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Verify Dashboard Per Role</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Verify that the admin lands on the admin dashboard</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>The admin admin is already in the system, nothing is made in the before step.</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as the admin</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>0799999999 and Irbid, Jordan, then 0791234567 and Amman, Jordan</t>
+          <t>admin / admin123</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>A toast reads "Profile saved." and the new phone and adress are shown, then the old ones are shown again.</t>
+          <t>The heading reads Admin Dashboard.</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
@@ -3807,27 +3804,27 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Verify that the admin lands on the admin dashboard</t>
+          <t>Verify that the doctor lands on the doctor dashboard</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>The admin admin is already in the system, nothing is made in the before step.</t>
+          <t>The doctor dr_smith is already in the system, nothing is made in the before step.</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as the admin</t>
+          <t>1. Log in as the doctor</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>admin / admin123</t>
+          <t>dr_smith / doctor123</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>The heading reads Admin Dashboard.</t>
+          <t>The heading reads Doctor Dashboard.</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr"/>
@@ -3851,27 +3848,27 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Verify that the doctor lands on the doctor dashboard</t>
+          <t>Verify that the patient lands on the patient dashboard</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>The doctor dr_smith is already in the system, nothing is made in the before step.</t>
+          <t>The patient john_doe is already in the system, nothing is made in the before step.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as the doctor</t>
+          <t>1. Log in as the patient</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>dr_smith / doctor123</t>
+          <t>john_doe / patient123</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>The heading reads Doctor Dashboard.</t>
+          <t>The heading reads My Dashboard.</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
@@ -3890,32 +3887,32 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Verify Dashboard Per Role</t>
+          <t>Verify Shared Profile</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Verify that the patient lands on the patient dashboard</t>
+          <t>Verify that an admin can not edit his own profile</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>The patient john_doe is already in the system, nothing is made in the before step.</t>
+          <t>The admin admin is logged in from the before step.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as the patient</t>
+          <t>1. Open the Profile page</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>john_doe / patient123</t>
+          <t>admin / admin123</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>The heading reads My Dashboard.</t>
+          <t>The page shows the username, says "An admin account is changed by another admin from the Admins page." and has no Edit Profile button.</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -3939,59 +3936,15 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Verify that an admin can not edit his own profile</t>
+          <t>Verify that the profile form does not save without a full name</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>The admin admin is logged in from the before step.</t>
+          <t>The patient john_doe is logged in from the before step.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Profile page</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>admin / admin123</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>The page shows the username, says "An admin account is changed by another admin from the Admins page." and has no Edit Profile button.</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77" ht="62" customHeight="1">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>TC-076</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Verify Shared Profile</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>Verify that the profile form does not save without a full name</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>The patient john_doe is logged in from the before step.</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>1. Open the Profile page
 2. Click Edit Profile
@@ -3999,14 +3952,59 @@
 4. Click Save Changes</t>
         </is>
       </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>An empty full name</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>The browser blocks the submit because the full name is required and the drawer stays open.</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77" ht="62" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>TC-076</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Verify Shared Settings</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Verify that the settings page shows who is signed in</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>The doctor dr_smith is logged in from the before step.</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Settings page
+2. Click Go to Profile</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>An empty full name</t>
+          <t>dr_smith / doctor123</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>The browser blocks the submit because the full name is required and the drawer stays open.</t>
+          <t>The settings page shows the username that is signed in and Go to Profile opens the profile page.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -4030,60 +4028,15 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Verify that the settings page shows who is signed in</t>
+          <t>Verify that a collapsed side menu is still collapsed after a reload</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>The doctor dr_smith is logged in from the before step.</t>
+          <t>The patient john_doe is logged in from the before step.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Settings page
-2. Click Go to Profile</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>dr_smith / doctor123</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>The settings page shows the username that is signed in and Go to Profile opens the profile page.</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
-    </row>
-    <row r="79" ht="62" customHeight="1">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>TC-078</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>Common</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>Verify Shared Settings</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>Verify that a collapsed side menu is still collapsed after a reload</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>The patient john_doe is logged in from the before step.</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>1. Open the Settings page
 2. Turn on Keep the side menu collapsed
@@ -4091,46 +4044,46 @@
 4. Turn it off again</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>No data</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>The side menu hides its labels while the switch is on, the switch is still on after the reload, and the labels come back when it is turned off.</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr"/>
-      <c r="J79" s="2" t="inlineStr"/>
-    </row>
-    <row r="80" ht="62" customHeight="1">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>TC-079</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79" ht="62" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>TC-078</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>Verify A Visit From Booking To Prescription</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>Verify that a booked visit can be completed and prescribed for and shows up in the record</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>The patient john_doe and the doctor dr_smith are already in the system. The appointment and the prescription the test needs are made by the test itself.</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>1. Log in as the patient and book an appointment
 2. Log in as the doctor, complete it and write a prescription
@@ -4138,21 +4091,21 @@
 4. Log in as the doctor and delete the prescription</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>Dr. Sarah Smith, a Monday eight weeks ahead, a reason and a diagnosis with unique numbers</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>The appointment turns Completed for the doctor, the prescription shows in the patient list and the visit shows as Completed in his record, and the prescription is removed at the end.</t>
-        </is>
-      </c>
-      <c r="I80" s="2" t="inlineStr"/>
-      <c r="J80" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>The appointment turns Completed for the doctor, the prescription shows in the patient list and the visit shows as Completed in his record, and the doctor can then change the diagnosis and delete the prescription.</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J80"/>
+  <autoFilter ref="A1:J79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test: let the visit test make its own patient and take him away after
Completing a visit can not be undone, so the appointment the test booked
stayed in the database for good. The admin makes a patient for the test
now and the after step deletes him, which takes his appointments with him.
</commit_message>
<xml_diff>
--- a/smart-healthcare-frontend/test-cases/test-cases.xlsx
+++ b/smart-healthcare-frontend/test-cases/test-cases.xlsx
@@ -4080,25 +4080,26 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>The patient john_doe and the doctor dr_smith are already in the system. The appointment and the prescription the test needs are made by the test itself.</t>
+          <t>The doctor dr_smith is already in the system. The admin makes a patient for this test in the before step, and the after step deletes him again with everything he booked.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>1. Log in as the patient and book an appointment
-2. Log in as the doctor, complete it and write a prescription
-3. Log in as the patient and read the prescription and the record
-4. Log in as the doctor and delete the prescription</t>
+          <t>1. Log in as the admin and add a patient
+2. Log in as that patient and book an appointment
+3. Log in as the doctor, complete it and write a prescription
+4. Log in as the patient and read the prescription and the record
+5. Log in as the doctor, change the diagnosis and delete the prescription</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Dr. Sarah Smith, a Monday eight weeks ahead, a reason and a diagnosis with unique numbers</t>
+          <t>A patient with a generated username, Dr. Sarah Smith, a Monday eight weeks ahead, a reason and a diagnosis with unique numbers</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>The appointment turns Completed for the doctor, the prescription shows in the patient list and the visit shows as Completed in his record, and the doctor can then change the diagnosis and delete the prescription.</t>
+          <t>The appointment turns Completed for the doctor, the prescription shows in the patient list and the visit shows as Completed in his record, the doctor can then change the diagnosis and delete the prescription, and deleting the patient takes his visit with him.</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>

</xml_diff>